<commit_message>
Real scraped product images (downloaded to docs/img, icon fallback); design docs as branded on-domain HTML pages; Vercel config
</commit_message>
<xml_diff>
--- a/data/incoming/stedman_products.xlsx
+++ b/data/incoming/stedman_products.xlsx
@@ -562,7 +562,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>https://img.source-werbeartikel.com/stedman/crusader.jpg</t>
+          <t>https://img.source-werbeartikel.com/media/catalog/product/cache/dc09e1c71e492175f875827bcbf6a37c/1/9/19809f56186701db0dcc101cf5b1bab9673d1198bc417d2dfa0646c6e0848d55.jpeg</t>
         </is>
       </c>
       <c r="M2" t="n">
@@ -640,7 +640,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>https://img.source-werbeartikel.com/stedman/iqoniq.jpg</t>
+          <t>https://img.source-werbeartikel.com/media/catalog/product/cache/dc09e1c71e492175f875827bcbf6a37c/0/4/04ea1f841899185842ba3c4d2beaf5c16c5306feec5f3d647e1da33145a69422.jpeg</t>
         </is>
       </c>
       <c r="M3" t="n">
@@ -718,7 +718,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>https://img.source-werbeartikel.com/stedman/monarch.jpg</t>
+          <t>https://img.source-werbeartikel.com/media/catalog/product/cache/dc09e1c71e492175f875827bcbf6a37c/7/c/7cf0207ebfd22ce9732b7b51e9bbbd3bb793024e99d6da9baa06bb506665b221.jpeg</t>
         </is>
       </c>
       <c r="M4" t="n">
@@ -794,7 +794,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>https://img.source-werbeartikel.com/stedman/legend.jpg</t>
+          <t>https://img.source-werbeartikel.com/media/catalog/product/cache/dc09e1c71e492175f875827bcbf6a37c/5/0/50a6e94bbb9aef327cce5db3fbfc0ca5348746dac7004dcbe9f894a595bff05b.jpeg</t>
         </is>
       </c>
       <c r="M5" t="n">
@@ -872,7 +872,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>https://img.source-werbeartikel.com/stedman/tuner.jpg</t>
+          <t>https://img.source-werbeartikel.com/media/catalog/product/cache/dc09e1c71e492175f875827bcbf6a37c/7/4/74d96df8083402a20c33b63df40a24751f82c82a9cd3466aa6c4c6ba14c687d3.jpeg</t>
         </is>
       </c>
       <c r="M6" t="n">

</xml_diff>